<commit_message>
Update PDS public dashboard/state: signal 2026-07, holding through 2026-08
</commit_message>
<xml_diff>
--- a/public/data/systems/pds/public_recent_12m_returns.xlsx
+++ b/public/data/systems/pds/public_recent_12m_returns.xlsx
@@ -48,7 +48,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Dynamic FX · 5bp</t>
+          <t>PDS + Dynamic FX (5bp)</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -79,13 +79,13 @@
         </is>
       </c>
       <c r="B2" s="1">
-        <v>0.02865984633458529</v>
+        <v>0.03480731918133273</v>
       </c>
       <c r="C2" s="1">
-        <v>0.05115615440670096</v>
+        <v>0.0574380695994956</v>
       </c>
       <c r="D2" s="1">
-        <v>0.07164132906138332</v>
+        <v>0.09694350871302371</v>
       </c>
       <c r="E2" s="1">
         <v>0.04437253533451946</v>
@@ -103,13 +103,13 @@
         </is>
       </c>
       <c r="B3" s="1">
-        <v>-0.06027352403745478</v>
+        <v>-0.05786895544144621</v>
       </c>
       <c r="C3" s="1">
-        <v>-0.05282400320937097</v>
+        <v>-0.05040037280729803</v>
       </c>
       <c r="D3" s="1">
-        <v>-0.0813899042759948</v>
+        <v>-0.07173192787694704</v>
       </c>
       <c r="E3" s="1">
         <v>-0.04327051572324403</v>
@@ -127,10 +127,10 @@
         </is>
       </c>
       <c r="B4" s="1">
-        <v>-0.006349162632413363</v>
+        <v>-0.006349162632414029</v>
       </c>
       <c r="C4" s="1">
-        <v>-0.02348466728004617</v>
+        <v>-0.02348466728004661</v>
       </c>
       <c r="D4" s="1">
         <v>-0.03191397779272764</v>
@@ -151,13 +151,13 @@
         </is>
       </c>
       <c r="B5" s="1">
-        <v>0.07552316304537787</v>
+        <v>0.07552316304537832</v>
       </c>
       <c r="C5" s="1">
-        <v>0.0680822510844179</v>
+        <v>0.06808225108441812</v>
       </c>
       <c r="D5" s="1">
-        <v>0.08241348173635243</v>
+        <v>0.08241348173635221</v>
       </c>
       <c r="E5" s="1">
         <v>0.06328153206946352</v>
@@ -175,13 +175,13 @@
         </is>
       </c>
       <c r="B6" s="1">
-        <v>0.08286669498855148</v>
+        <v>0.08283399502926669</v>
       </c>
       <c r="C6" s="1">
-        <v>0.09369335078245644</v>
+        <v>0.09366032388431056</v>
       </c>
       <c r="D6" s="1">
-        <v>0.138116221557653</v>
+        <v>0.1379985506159107</v>
       </c>
       <c r="E6" s="1">
         <v>0.07894707047686933</v>
@@ -199,13 +199,13 @@
         </is>
       </c>
       <c r="B7" s="1">
-        <v>-0.05292396020991308</v>
+        <v>-0.0525388215458209</v>
       </c>
       <c r="C7" s="1">
-        <v>-0.07554630879154212</v>
+        <v>-0.07517036974896418</v>
       </c>
       <c r="D7" s="1">
-        <v>-0.08804818870189246</v>
+        <v>-0.0864924086562967</v>
       </c>
       <c r="E7" s="1">
         <v>-0.07137572261430858</v>
@@ -223,13 +223,13 @@
         </is>
       </c>
       <c r="B8" s="1">
-        <v>0.04855655795233171</v>
+        <v>0.05355636201714331</v>
       </c>
       <c r="C8" s="1">
-        <v>0.04750981875209215</v>
+        <v>0.05250463167849762</v>
       </c>
       <c r="D8" s="1">
-        <v>0.008834524013307865</v>
+        <v>0.02882602930971068</v>
       </c>
       <c r="E8" s="1">
         <v>0.06040569932885687</v>
@@ -247,13 +247,13 @@
         </is>
       </c>
       <c r="B9" s="1">
-        <v>0.07073007740498083</v>
+        <v>0.07131811233513297</v>
       </c>
       <c r="C9" s="1">
-        <v>0.07442562966675537</v>
+        <v>0.07501569415959697</v>
       </c>
       <c r="D9" s="1">
-        <v>0.06745922795148496</v>
+        <v>0.06981911240614602</v>
       </c>
       <c r="E9" s="1">
         <v>0.07672064779432697</v>
@@ -271,13 +271,13 @@
         </is>
       </c>
       <c r="B10" s="1">
-        <v>0.01172031519172112</v>
+        <v>0.01172032135908996</v>
       </c>
       <c r="C10" s="1">
-        <v>0.0201407739614734</v>
+        <v>0.02014078018017185</v>
       </c>
       <c r="D10" s="1">
-        <v>0.02426738196587452</v>
+        <v>0.02426740697417418</v>
       </c>
       <c r="E10" s="1">
         <v>0.01875736131405326</v>
@@ -295,13 +295,13 @@
         </is>
       </c>
       <c r="B11" s="1">
-        <v>0.01148210469120681</v>
+        <v>0.01166436280053529</v>
       </c>
       <c r="C11" s="1">
-        <v>-0.001367367880744985</v>
+        <v>-0.001187425107066598</v>
       </c>
       <c r="D11" s="1">
-        <v>-0.005218051108377031</v>
+        <v>-0.004492457278143069</v>
       </c>
       <c r="E11" s="1">
         <v>-8.422169188504469e-05</v>
@@ -319,13 +319,13 @@
         </is>
       </c>
       <c r="B12" s="1">
-        <v>0.04945256734711112</v>
+        <v>0.05056190453239551</v>
       </c>
       <c r="C12" s="1">
-        <v>0.04196369833249625</v>
+        <v>0.04306511931353163</v>
       </c>
       <c r="D12" s="1">
-        <v>0.03462977045244275</v>
+        <v>0.03904012692536307</v>
       </c>
       <c r="E12" s="1">
         <v>0.044410290250674</v>
@@ -343,13 +343,13 @@
         </is>
       </c>
       <c r="B13" s="1">
-        <v>0.07400328952065482</v>
+        <v>0.07355902411024573</v>
       </c>
       <c r="C13" s="1">
-        <v>0.06707176895797518</v>
+        <v>0.06663037079653833</v>
       </c>
       <c r="D13" s="1">
-        <v>0.08054512040851125</v>
+        <v>0.07878106091421655</v>
       </c>
       <c r="E13" s="1">
         <v>0.06259113492093893</v>
@@ -387,7 +387,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>F2R 25% + ADAA 75% fixed over displayed history</t>
+          <t>Governed strategic allocation; exact provider composition private</t>
         </is>
       </c>
     </row>
@@ -423,7 +423,19 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SlackQuant PDS public-safe governed export</t>
+          <t>Source-owned PDS public-safe governed export</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CSV SHA256</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>d527da8625755b4774c7423c97275c86e56dd3fbd0960e5d9962779502e420ba</t>
         </is>
       </c>
     </row>

</xml_diff>